<commit_message>
V4: Use Trade ID for deduplication instead of Symbol+Date+Price matching
</commit_message>
<xml_diff>
--- a/Tradebook Template - Copy.xlsx
+++ b/Tradebook Template - Copy.xlsx
@@ -3,13 +3,16 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28925"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="5" documentId="11_B8E6E54BA230E35AD1C0AFADF073B256A24125FE" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9D1DF9AC-7901-4E7D-A289-13DEB17295FC}"/>
+  <xr:revisionPtr revIDLastSave="10" documentId="11_B8E6E54BA230E35AD1C0AFADF073B256A24125FE" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4A05C565-BA66-46C1-8093-5EBB7AA3656F}"/>
   <bookViews>
-    <workbookView minimized="1" xWindow="2415" yWindow="2415" windowWidth="2400" windowHeight="585" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView minimized="1" xWindow="3105" yWindow="3105" windowWidth="2400" windowHeight="585" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Equity" sheetId="1" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Equity!$B$1:$N$363</definedName>
+  </definedNames>
   <calcPr calcId="122211"/>
 </workbook>
 </file>
@@ -2336,7 +2339,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -2344,6 +2347,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2359,10 +2363,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2623,7 +2623,8 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="B1:N363"/>
+  <sheetPr filterMode="1"/>
+  <dimension ref="B1:N374"/>
   <sheetFormatPr defaultColWidth="15" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="2" customWidth="1"/>
@@ -2673,7 +2674,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="2" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="2" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B2" t="s">
         <v>17</v>
       </c>
@@ -2755,7 +2756,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="4" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B4" t="s">
         <v>29</v>
       </c>
@@ -2796,7 +2797,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="5" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B5" t="s">
         <v>29</v>
       </c>
@@ -2837,7 +2838,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="6" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B6" t="s">
         <v>29</v>
       </c>
@@ -2878,7 +2879,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="7" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B7" t="s">
         <v>29</v>
       </c>
@@ -2960,7 +2961,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="9" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B9" t="s">
         <v>42</v>
       </c>
@@ -3001,7 +3002,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="10" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B10" t="s">
         <v>42</v>
       </c>
@@ -3042,7 +3043,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="11" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="11" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B11" t="s">
         <v>48</v>
       </c>
@@ -3083,7 +3084,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="12" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="12" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B12" t="s">
         <v>48</v>
       </c>
@@ -3124,7 +3125,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="13" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="13" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B13" t="s">
         <v>48</v>
       </c>
@@ -3165,7 +3166,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="14" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="14" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B14" t="s">
         <v>48</v>
       </c>
@@ -3206,7 +3207,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="15" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="15" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B15" t="s">
         <v>56</v>
       </c>
@@ -3247,7 +3248,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="16" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="16" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B16" t="s">
         <v>61</v>
       </c>
@@ -3288,7 +3289,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="17" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B17" t="s">
         <v>61</v>
       </c>
@@ -3329,7 +3330,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="18" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B18" t="s">
         <v>61</v>
       </c>
@@ -3370,7 +3371,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="19" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="19" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B19" t="s">
         <v>69</v>
       </c>
@@ -3411,7 +3412,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="20" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="20" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B20" t="s">
         <v>69</v>
       </c>
@@ -3452,7 +3453,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="21" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="21" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B21" t="s">
         <v>69</v>
       </c>
@@ -3493,7 +3494,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="22" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="22" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B22" t="s">
         <v>69</v>
       </c>
@@ -3534,7 +3535,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="23" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="23" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B23" t="s">
         <v>77</v>
       </c>
@@ -3575,7 +3576,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="24" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="24" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B24" t="s">
         <v>77</v>
       </c>
@@ -3616,7 +3617,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="25" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="25" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B25" t="s">
         <v>77</v>
       </c>
@@ -3657,7 +3658,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="26" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="26" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B26" t="s">
         <v>77</v>
       </c>
@@ -3698,7 +3699,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="27" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="27" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B27" t="s">
         <v>77</v>
       </c>
@@ -3739,7 +3740,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="28" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="28" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B28" t="s">
         <v>77</v>
       </c>
@@ -3780,7 +3781,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="29" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="29" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B29" t="s">
         <v>77</v>
       </c>
@@ -3821,7 +3822,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="30" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="30" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B30" t="s">
         <v>88</v>
       </c>
@@ -3862,7 +3863,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="31" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="31" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B31" t="s">
         <v>93</v>
       </c>
@@ -3903,7 +3904,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="32" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="32" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B32" t="s">
         <v>93</v>
       </c>
@@ -3944,7 +3945,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="33" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="33" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B33" t="s">
         <v>100</v>
       </c>
@@ -3985,7 +3986,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="34" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="34" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B34" t="s">
         <v>106</v>
       </c>
@@ -4026,7 +4027,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="35" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="35" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B35" t="s">
         <v>106</v>
       </c>
@@ -4067,7 +4068,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="36" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="36" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B36" t="s">
         <v>106</v>
       </c>
@@ -4108,7 +4109,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="37" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="37" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B37" t="s">
         <v>61</v>
       </c>
@@ -4149,7 +4150,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="38" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="38" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B38" t="s">
         <v>61</v>
       </c>
@@ -4190,7 +4191,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="39" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="39" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B39" t="s">
         <v>61</v>
       </c>
@@ -4231,7 +4232,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="40" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="40" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B40" t="s">
         <v>69</v>
       </c>
@@ -4272,7 +4273,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="41" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="41" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B41" t="s">
         <v>69</v>
       </c>
@@ -4313,7 +4314,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="42" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="42" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B42" t="s">
         <v>123</v>
       </c>
@@ -4354,7 +4355,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="43" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="43" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B43" t="s">
         <v>123</v>
       </c>
@@ -4395,7 +4396,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="44" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="44" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B44" t="s">
         <v>123</v>
       </c>
@@ -4436,7 +4437,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="45" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="45" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B45" t="s">
         <v>42</v>
       </c>
@@ -4477,7 +4478,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="46" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="46" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B46" t="s">
         <v>42</v>
       </c>
@@ -4518,7 +4519,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="47" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="47" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B47" t="s">
         <v>42</v>
       </c>
@@ -4559,7 +4560,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="48" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="48" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B48" t="s">
         <v>42</v>
       </c>
@@ -4928,7 +4929,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="57" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="57" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B57" t="s">
         <v>88</v>
       </c>
@@ -4969,7 +4970,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="58" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="58" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B58" t="s">
         <v>88</v>
       </c>
@@ -5010,7 +5011,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="59" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="59" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B59" t="s">
         <v>88</v>
       </c>
@@ -5051,7 +5052,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="60" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="60" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B60" t="s">
         <v>88</v>
       </c>
@@ -5092,7 +5093,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="61" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="61" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B61" t="s">
         <v>88</v>
       </c>
@@ -5133,7 +5134,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="62" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="62" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B62" t="s">
         <v>88</v>
       </c>
@@ -5174,7 +5175,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="63" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="63" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B63" t="s">
         <v>88</v>
       </c>
@@ -5215,7 +5216,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="64" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="64" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B64" t="s">
         <v>88</v>
       </c>
@@ -5256,7 +5257,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="65" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="65" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B65" t="s">
         <v>88</v>
       </c>
@@ -5297,7 +5298,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="66" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="66" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B66" t="s">
         <v>88</v>
       </c>
@@ -5338,7 +5339,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="67" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="67" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B67" t="s">
         <v>88</v>
       </c>
@@ -5379,7 +5380,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="68" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="68" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B68" t="s">
         <v>106</v>
       </c>
@@ -5420,7 +5421,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="69" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="69" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B69" t="s">
         <v>106</v>
       </c>
@@ -5461,7 +5462,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="70" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="70" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B70" t="s">
         <v>106</v>
       </c>
@@ -5502,7 +5503,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="71" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="71" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B71" t="s">
         <v>106</v>
       </c>
@@ -5543,7 +5544,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="72" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="72" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B72" t="s">
         <v>106</v>
       </c>
@@ -5584,7 +5585,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="73" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="73" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B73" t="s">
         <v>106</v>
       </c>
@@ -5625,7 +5626,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="74" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="74" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B74" t="s">
         <v>106</v>
       </c>
@@ -5666,7 +5667,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="75" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="75" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B75" t="s">
         <v>106</v>
       </c>
@@ -5707,7 +5708,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="76" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="76" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B76" t="s">
         <v>106</v>
       </c>
@@ -5748,7 +5749,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="77" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="77" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B77" t="s">
         <v>106</v>
       </c>
@@ -5789,7 +5790,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="78" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="78" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B78" t="s">
         <v>106</v>
       </c>
@@ -5830,7 +5831,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="79" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="79" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B79" t="s">
         <v>106</v>
       </c>
@@ -5871,7 +5872,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="80" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="80" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B80" t="s">
         <v>106</v>
       </c>
@@ -5912,7 +5913,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="81" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="81" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B81" t="s">
         <v>106</v>
       </c>
@@ -5953,7 +5954,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="82" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="82" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B82" t="s">
         <v>106</v>
       </c>
@@ -5994,7 +5995,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="83" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="83" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B83" t="s">
         <v>106</v>
       </c>
@@ -6035,7 +6036,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="84" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="84" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B84" t="s">
         <v>106</v>
       </c>
@@ -6076,7 +6077,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="85" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="85" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B85" t="s">
         <v>106</v>
       </c>
@@ -6117,7 +6118,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="86" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="86" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B86" t="s">
         <v>106</v>
       </c>
@@ -6158,7 +6159,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="87" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="87" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B87" t="s">
         <v>106</v>
       </c>
@@ -6199,7 +6200,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="88" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="88" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B88" t="s">
         <v>61</v>
       </c>
@@ -6240,7 +6241,7 @@
         <v>188</v>
       </c>
     </row>
-    <row r="89" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="89" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B89" t="s">
         <v>189</v>
       </c>
@@ -6281,7 +6282,7 @@
         <v>193</v>
       </c>
     </row>
-    <row r="90" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="90" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B90" t="s">
         <v>189</v>
       </c>
@@ -6322,7 +6323,7 @@
         <v>193</v>
       </c>
     </row>
-    <row r="91" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="91" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B91" t="s">
         <v>189</v>
       </c>
@@ -6363,7 +6364,7 @@
         <v>193</v>
       </c>
     </row>
-    <row r="92" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="92" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B92" t="s">
         <v>196</v>
       </c>
@@ -6404,7 +6405,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="93" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="93" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B93" t="s">
         <v>196</v>
       </c>
@@ -6445,7 +6446,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="94" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="94" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B94" t="s">
         <v>196</v>
       </c>
@@ -6486,7 +6487,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="95" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="95" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B95" t="s">
         <v>196</v>
       </c>
@@ -6527,7 +6528,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="96" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="96" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B96" t="s">
         <v>196</v>
       </c>
@@ -6568,7 +6569,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="97" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="97" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B97" t="s">
         <v>196</v>
       </c>
@@ -6609,7 +6610,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="98" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="98" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B98" t="s">
         <v>196</v>
       </c>
@@ -6650,7 +6651,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="99" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="99" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B99" t="s">
         <v>196</v>
       </c>
@@ -6691,7 +6692,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="100" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="100" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B100" t="s">
         <v>196</v>
       </c>
@@ -6732,7 +6733,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="101" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="101" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B101" t="s">
         <v>196</v>
       </c>
@@ -6773,7 +6774,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="102" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="102" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B102" t="s">
         <v>196</v>
       </c>
@@ -6814,7 +6815,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="103" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="103" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B103" t="s">
         <v>196</v>
       </c>
@@ -6855,7 +6856,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="104" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="104" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B104" t="s">
         <v>196</v>
       </c>
@@ -6896,7 +6897,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="105" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="105" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B105" t="s">
         <v>196</v>
       </c>
@@ -6937,7 +6938,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="106" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="106" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B106" t="s">
         <v>196</v>
       </c>
@@ -6978,7 +6979,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="107" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="107" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B107" t="s">
         <v>196</v>
       </c>
@@ -7019,7 +7020,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="108" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="108" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B108" t="s">
         <v>196</v>
       </c>
@@ -7060,7 +7061,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="109" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="109" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B109" t="s">
         <v>196</v>
       </c>
@@ -7101,7 +7102,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="110" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="110" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B110" t="s">
         <v>196</v>
       </c>
@@ -7142,7 +7143,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="111" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="111" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B111" t="s">
         <v>196</v>
       </c>
@@ -7183,7 +7184,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="112" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="112" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B112" t="s">
         <v>196</v>
       </c>
@@ -7224,7 +7225,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="113" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="113" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B113" t="s">
         <v>196</v>
       </c>
@@ -7265,7 +7266,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="114" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="114" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B114" t="s">
         <v>196</v>
       </c>
@@ -7306,7 +7307,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="115" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="115" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B115" t="s">
         <v>69</v>
       </c>
@@ -7347,7 +7348,7 @@
         <v>225</v>
       </c>
     </row>
-    <row r="116" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="116" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B116" t="s">
         <v>226</v>
       </c>
@@ -7388,7 +7389,7 @@
         <v>230</v>
       </c>
     </row>
-    <row r="117" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="117" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B117" t="s">
         <v>226</v>
       </c>
@@ -7429,7 +7430,7 @@
         <v>230</v>
       </c>
     </row>
-    <row r="118" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="118" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B118" t="s">
         <v>123</v>
       </c>
@@ -7470,7 +7471,7 @@
         <v>235</v>
       </c>
     </row>
-    <row r="119" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="119" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B119" t="s">
         <v>123</v>
       </c>
@@ -7511,7 +7512,7 @@
         <v>235</v>
       </c>
     </row>
-    <row r="120" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="120" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B120" t="s">
         <v>123</v>
       </c>
@@ -7552,7 +7553,7 @@
         <v>235</v>
       </c>
     </row>
-    <row r="121" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="121" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B121" t="s">
         <v>123</v>
       </c>
@@ -7593,7 +7594,7 @@
         <v>235</v>
       </c>
     </row>
-    <row r="122" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="122" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B122" t="s">
         <v>123</v>
       </c>
@@ -7634,7 +7635,7 @@
         <v>235</v>
       </c>
     </row>
-    <row r="123" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="123" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B123" t="s">
         <v>123</v>
       </c>
@@ -7675,7 +7676,7 @@
         <v>235</v>
       </c>
     </row>
-    <row r="124" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="124" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B124" t="s">
         <v>123</v>
       </c>
@@ -7716,7 +7717,7 @@
         <v>235</v>
       </c>
     </row>
-    <row r="125" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="125" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B125" t="s">
         <v>123</v>
       </c>
@@ -7757,7 +7758,7 @@
         <v>235</v>
       </c>
     </row>
-    <row r="126" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="126" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B126" t="s">
         <v>123</v>
       </c>
@@ -7798,7 +7799,7 @@
         <v>235</v>
       </c>
     </row>
-    <row r="127" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="127" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B127" t="s">
         <v>17</v>
       </c>
@@ -7839,7 +7840,7 @@
         <v>247</v>
       </c>
     </row>
-    <row r="128" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="128" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B128" t="s">
         <v>106</v>
       </c>
@@ -7880,7 +7881,7 @@
         <v>251</v>
       </c>
     </row>
-    <row r="129" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="129" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B129" t="s">
         <v>106</v>
       </c>
@@ -7921,7 +7922,7 @@
         <v>251</v>
       </c>
     </row>
-    <row r="130" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="130" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B130" t="s">
         <v>61</v>
       </c>
@@ -7962,7 +7963,7 @@
         <v>255</v>
       </c>
     </row>
-    <row r="131" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="131" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B131" t="s">
         <v>61</v>
       </c>
@@ -8003,7 +8004,7 @@
         <v>255</v>
       </c>
     </row>
-    <row r="132" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="132" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B132" t="s">
         <v>257</v>
       </c>
@@ -8044,7 +8045,7 @@
         <v>262</v>
       </c>
     </row>
-    <row r="133" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="133" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B133" t="s">
         <v>257</v>
       </c>
@@ -8085,7 +8086,7 @@
         <v>262</v>
       </c>
     </row>
-    <row r="134" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="134" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B134" t="s">
         <v>257</v>
       </c>
@@ -8126,7 +8127,7 @@
         <v>262</v>
       </c>
     </row>
-    <row r="135" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="135" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B135" t="s">
         <v>257</v>
       </c>
@@ -8167,7 +8168,7 @@
         <v>262</v>
       </c>
     </row>
-    <row r="136" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="136" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B136" t="s">
         <v>29</v>
       </c>
@@ -8208,7 +8209,7 @@
         <v>268</v>
       </c>
     </row>
-    <row r="137" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="137" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B137" t="s">
         <v>93</v>
       </c>
@@ -8249,7 +8250,7 @@
         <v>272</v>
       </c>
     </row>
-    <row r="138" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="138" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B138" t="s">
         <v>93</v>
       </c>
@@ -8290,7 +8291,7 @@
         <v>272</v>
       </c>
     </row>
-    <row r="139" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="139" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B139" t="s">
         <v>100</v>
       </c>
@@ -8331,7 +8332,7 @@
         <v>276</v>
       </c>
     </row>
-    <row r="140" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="140" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B140" t="s">
         <v>100</v>
       </c>
@@ -8372,7 +8373,7 @@
         <v>276</v>
       </c>
     </row>
-    <row r="141" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="141" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B141" t="s">
         <v>61</v>
       </c>
@@ -8413,7 +8414,7 @@
         <v>281</v>
       </c>
     </row>
-    <row r="142" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="142" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B142" t="s">
         <v>61</v>
       </c>
@@ -8454,7 +8455,7 @@
         <v>281</v>
       </c>
     </row>
-    <row r="143" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="143" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B143" t="s">
         <v>61</v>
       </c>
@@ -8495,7 +8496,7 @@
         <v>281</v>
       </c>
     </row>
-    <row r="144" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="144" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B144" t="s">
         <v>284</v>
       </c>
@@ -8536,7 +8537,7 @@
         <v>289</v>
       </c>
     </row>
-    <row r="145" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="145" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B145" t="s">
         <v>106</v>
       </c>
@@ -8577,7 +8578,7 @@
         <v>292</v>
       </c>
     </row>
-    <row r="146" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="146" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B146" t="s">
         <v>69</v>
       </c>
@@ -8618,7 +8619,7 @@
         <v>296</v>
       </c>
     </row>
-    <row r="147" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="147" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B147" t="s">
         <v>69</v>
       </c>
@@ -8659,7 +8660,7 @@
         <v>296</v>
       </c>
     </row>
-    <row r="148" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="148" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B148" t="s">
         <v>69</v>
       </c>
@@ -8700,7 +8701,7 @@
         <v>296</v>
       </c>
     </row>
-    <row r="149" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="149" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B149" t="s">
         <v>69</v>
       </c>
@@ -8741,7 +8742,7 @@
         <v>296</v>
       </c>
     </row>
-    <row r="150" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="150" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B150" t="s">
         <v>69</v>
       </c>
@@ -8782,7 +8783,7 @@
         <v>296</v>
       </c>
     </row>
-    <row r="151" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="151" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B151" t="s">
         <v>69</v>
       </c>
@@ -8823,7 +8824,7 @@
         <v>296</v>
       </c>
     </row>
-    <row r="152" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="152" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B152" t="s">
         <v>69</v>
       </c>
@@ -8864,7 +8865,7 @@
         <v>296</v>
       </c>
     </row>
-    <row r="153" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="153" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B153" t="s">
         <v>189</v>
       </c>
@@ -8905,7 +8906,7 @@
         <v>306</v>
       </c>
     </row>
-    <row r="154" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="154" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B154" t="s">
         <v>189</v>
       </c>
@@ -8946,7 +8947,7 @@
         <v>306</v>
       </c>
     </row>
-    <row r="155" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="155" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B155" t="s">
         <v>189</v>
       </c>
@@ -8987,7 +8988,7 @@
         <v>306</v>
       </c>
     </row>
-    <row r="156" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="156" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B156" t="s">
         <v>189</v>
       </c>
@@ -9028,7 +9029,7 @@
         <v>306</v>
       </c>
     </row>
-    <row r="157" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="157" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B157" t="s">
         <v>189</v>
       </c>
@@ -9069,7 +9070,7 @@
         <v>306</v>
       </c>
     </row>
-    <row r="158" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="158" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B158" t="s">
         <v>189</v>
       </c>
@@ -9110,7 +9111,7 @@
         <v>306</v>
       </c>
     </row>
-    <row r="159" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="159" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B159" t="s">
         <v>189</v>
       </c>
@@ -9151,7 +9152,7 @@
         <v>306</v>
       </c>
     </row>
-    <row r="160" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="160" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B160" t="s">
         <v>189</v>
       </c>
@@ -9192,7 +9193,7 @@
         <v>306</v>
       </c>
     </row>
-    <row r="161" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="161" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B161" t="s">
         <v>189</v>
       </c>
@@ -9233,7 +9234,7 @@
         <v>306</v>
       </c>
     </row>
-    <row r="162" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="162" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B162" t="s">
         <v>189</v>
       </c>
@@ -9274,7 +9275,7 @@
         <v>306</v>
       </c>
     </row>
-    <row r="163" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="163" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B163" t="s">
         <v>189</v>
       </c>
@@ -9315,7 +9316,7 @@
         <v>306</v>
       </c>
     </row>
-    <row r="164" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="164" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B164" t="s">
         <v>189</v>
       </c>
@@ -9356,7 +9357,7 @@
         <v>306</v>
       </c>
     </row>
-    <row r="165" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="165" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B165" t="s">
         <v>189</v>
       </c>
@@ -9397,7 +9398,7 @@
         <v>306</v>
       </c>
     </row>
-    <row r="166" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="166" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B166" t="s">
         <v>189</v>
       </c>
@@ -9438,7 +9439,7 @@
         <v>306</v>
       </c>
     </row>
-    <row r="167" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="167" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B167" t="s">
         <v>189</v>
       </c>
@@ -9479,7 +9480,7 @@
         <v>306</v>
       </c>
     </row>
-    <row r="168" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="168" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B168" t="s">
         <v>189</v>
       </c>
@@ -9520,7 +9521,7 @@
         <v>306</v>
       </c>
     </row>
-    <row r="169" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="169" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B169" t="s">
         <v>226</v>
       </c>
@@ -9561,7 +9562,7 @@
         <v>324</v>
       </c>
     </row>
-    <row r="170" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="170" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B170" t="s">
         <v>226</v>
       </c>
@@ -9602,7 +9603,7 @@
         <v>324</v>
       </c>
     </row>
-    <row r="171" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="171" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B171" t="s">
         <v>326</v>
       </c>
@@ -9643,7 +9644,7 @@
         <v>330</v>
       </c>
     </row>
-    <row r="172" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="172" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B172" t="s">
         <v>326</v>
       </c>
@@ -9684,7 +9685,7 @@
         <v>330</v>
       </c>
     </row>
-    <row r="173" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="173" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B173" t="s">
         <v>326</v>
       </c>
@@ -9725,7 +9726,7 @@
         <v>335</v>
       </c>
     </row>
-    <row r="174" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="174" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B174" t="s">
         <v>326</v>
       </c>
@@ -9766,7 +9767,7 @@
         <v>335</v>
       </c>
     </row>
-    <row r="175" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="175" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B175" t="s">
         <v>337</v>
       </c>
@@ -9807,7 +9808,7 @@
         <v>342</v>
       </c>
     </row>
-    <row r="176" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="176" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B176" t="s">
         <v>337</v>
       </c>
@@ -9848,7 +9849,7 @@
         <v>342</v>
       </c>
     </row>
-    <row r="177" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="177" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B177" t="s">
         <v>337</v>
       </c>
@@ -9889,7 +9890,7 @@
         <v>342</v>
       </c>
     </row>
-    <row r="178" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="178" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B178" t="s">
         <v>345</v>
       </c>
@@ -9930,7 +9931,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="179" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="179" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B179" t="s">
         <v>345</v>
       </c>
@@ -9971,7 +9972,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="180" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="180" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B180" t="s">
         <v>345</v>
       </c>
@@ -10012,7 +10013,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="181" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="181" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B181" t="s">
         <v>345</v>
       </c>
@@ -10053,7 +10054,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="182" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="182" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B182" t="s">
         <v>345</v>
       </c>
@@ -10094,7 +10095,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="183" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="183" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B183" t="s">
         <v>345</v>
       </c>
@@ -10135,7 +10136,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="184" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="184" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B184" t="s">
         <v>355</v>
       </c>
@@ -10176,7 +10177,7 @@
         <v>359</v>
       </c>
     </row>
-    <row r="185" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="185" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B185" t="s">
         <v>360</v>
       </c>
@@ -10217,7 +10218,7 @@
         <v>364</v>
       </c>
     </row>
-    <row r="186" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="186" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B186" t="s">
         <v>360</v>
       </c>
@@ -10258,7 +10259,7 @@
         <v>364</v>
       </c>
     </row>
-    <row r="187" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="187" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B187" t="s">
         <v>366</v>
       </c>
@@ -10299,7 +10300,7 @@
         <v>370</v>
       </c>
     </row>
-    <row r="188" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="188" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B188" t="s">
         <v>366</v>
       </c>
@@ -10340,7 +10341,7 @@
         <v>370</v>
       </c>
     </row>
-    <row r="189" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="189" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B189" t="s">
         <v>366</v>
       </c>
@@ -10381,7 +10382,7 @@
         <v>370</v>
       </c>
     </row>
-    <row r="190" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="190" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B190" t="s">
         <v>366</v>
       </c>
@@ -10422,7 +10423,7 @@
         <v>370</v>
       </c>
     </row>
-    <row r="191" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="191" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B191" t="s">
         <v>366</v>
       </c>
@@ -10463,7 +10464,7 @@
         <v>370</v>
       </c>
     </row>
-    <row r="192" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="192" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B192" t="s">
         <v>366</v>
       </c>
@@ -10504,7 +10505,7 @@
         <v>370</v>
       </c>
     </row>
-    <row r="193" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="193" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B193" t="s">
         <v>366</v>
       </c>
@@ -10545,7 +10546,7 @@
         <v>370</v>
       </c>
     </row>
-    <row r="194" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="194" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B194" t="s">
         <v>366</v>
       </c>
@@ -10586,7 +10587,7 @@
         <v>370</v>
       </c>
     </row>
-    <row r="195" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="195" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B195" t="s">
         <v>366</v>
       </c>
@@ -10627,7 +10628,7 @@
         <v>370</v>
       </c>
     </row>
-    <row r="196" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="196" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B196" t="s">
         <v>366</v>
       </c>
@@ -10668,7 +10669,7 @@
         <v>370</v>
       </c>
     </row>
-    <row r="197" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="197" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B197" t="s">
         <v>366</v>
       </c>
@@ -10709,7 +10710,7 @@
         <v>370</v>
       </c>
     </row>
-    <row r="198" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="198" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B198" t="s">
         <v>366</v>
       </c>
@@ -10750,7 +10751,7 @@
         <v>370</v>
       </c>
     </row>
-    <row r="199" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="199" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B199" t="s">
         <v>366</v>
       </c>
@@ -10791,7 +10792,7 @@
         <v>370</v>
       </c>
     </row>
-    <row r="200" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="200" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B200" t="s">
         <v>366</v>
       </c>
@@ -10832,7 +10833,7 @@
         <v>370</v>
       </c>
     </row>
-    <row r="201" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="201" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B201" t="s">
         <v>366</v>
       </c>
@@ -10873,7 +10874,7 @@
         <v>370</v>
       </c>
     </row>
-    <row r="202" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="202" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B202" t="s">
         <v>366</v>
       </c>
@@ -10914,7 +10915,7 @@
         <v>370</v>
       </c>
     </row>
-    <row r="203" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="203" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B203" t="s">
         <v>366</v>
       </c>
@@ -10955,7 +10956,7 @@
         <v>370</v>
       </c>
     </row>
-    <row r="204" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="204" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B204" t="s">
         <v>366</v>
       </c>
@@ -10996,7 +10997,7 @@
         <v>370</v>
       </c>
     </row>
-    <row r="205" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="205" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B205" t="s">
         <v>366</v>
       </c>
@@ -11037,7 +11038,7 @@
         <v>370</v>
       </c>
     </row>
-    <row r="206" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="206" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B206" t="s">
         <v>366</v>
       </c>
@@ -11078,7 +11079,7 @@
         <v>370</v>
       </c>
     </row>
-    <row r="207" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="207" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B207" t="s">
         <v>366</v>
       </c>
@@ -11119,7 +11120,7 @@
         <v>370</v>
       </c>
     </row>
-    <row r="208" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="208" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B208" t="s">
         <v>366</v>
       </c>
@@ -11160,7 +11161,7 @@
         <v>370</v>
       </c>
     </row>
-    <row r="209" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="209" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B209" t="s">
         <v>366</v>
       </c>
@@ -11201,7 +11202,7 @@
         <v>370</v>
       </c>
     </row>
-    <row r="210" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="210" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B210" t="s">
         <v>366</v>
       </c>
@@ -11242,7 +11243,7 @@
         <v>370</v>
       </c>
     </row>
-    <row r="211" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="211" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B211" t="s">
         <v>366</v>
       </c>
@@ -11283,7 +11284,7 @@
         <v>370</v>
       </c>
     </row>
-    <row r="212" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="212" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B212" t="s">
         <v>395</v>
       </c>
@@ -11324,7 +11325,7 @@
         <v>399</v>
       </c>
     </row>
-    <row r="213" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="213" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B213" t="s">
         <v>400</v>
       </c>
@@ -11365,7 +11366,7 @@
         <v>404</v>
       </c>
     </row>
-    <row r="214" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="214" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B214" t="s">
         <v>400</v>
       </c>
@@ -11406,7 +11407,7 @@
         <v>404</v>
       </c>
     </row>
-    <row r="215" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="215" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B215" t="s">
         <v>400</v>
       </c>
@@ -11447,7 +11448,7 @@
         <v>404</v>
       </c>
     </row>
-    <row r="216" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="216" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B216" t="s">
         <v>284</v>
       </c>
@@ -11488,7 +11489,7 @@
         <v>410</v>
       </c>
     </row>
-    <row r="217" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="217" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B217" t="s">
         <v>284</v>
       </c>
@@ -11529,7 +11530,7 @@
         <v>410</v>
       </c>
     </row>
-    <row r="218" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="218" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B218" t="s">
         <v>284</v>
       </c>
@@ -11570,7 +11571,7 @@
         <v>410</v>
       </c>
     </row>
-    <row r="219" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="219" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B219" t="s">
         <v>48</v>
       </c>
@@ -11611,7 +11612,7 @@
         <v>416</v>
       </c>
     </row>
-    <row r="220" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="220" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B220" t="s">
         <v>56</v>
       </c>
@@ -11652,7 +11653,7 @@
         <v>419</v>
       </c>
     </row>
-    <row r="221" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="221" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B221" t="s">
         <v>56</v>
       </c>
@@ -11693,7 +11694,7 @@
         <v>419</v>
       </c>
     </row>
-    <row r="222" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="222" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B222" t="s">
         <v>17</v>
       </c>
@@ -11734,7 +11735,7 @@
         <v>424</v>
       </c>
     </row>
-    <row r="223" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="223" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B223" t="s">
         <v>17</v>
       </c>
@@ -11775,7 +11776,7 @@
         <v>424</v>
       </c>
     </row>
-    <row r="224" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="224" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B224" t="s">
         <v>17</v>
       </c>
@@ -11816,7 +11817,7 @@
         <v>424</v>
       </c>
     </row>
-    <row r="225" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="225" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B225" t="s">
         <v>17</v>
       </c>
@@ -11857,7 +11858,7 @@
         <v>424</v>
       </c>
     </row>
-    <row r="226" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="226" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B226" t="s">
         <v>17</v>
       </c>
@@ -11898,7 +11899,7 @@
         <v>424</v>
       </c>
     </row>
-    <row r="227" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="227" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B227" t="s">
         <v>17</v>
       </c>
@@ -11939,7 +11940,7 @@
         <v>424</v>
       </c>
     </row>
-    <row r="228" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="228" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B228" t="s">
         <v>196</v>
       </c>
@@ -11980,7 +11981,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="229" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="229" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B229" t="s">
         <v>196</v>
       </c>
@@ -12021,7 +12022,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="230" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="230" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B230" t="s">
         <v>435</v>
       </c>
@@ -12062,7 +12063,7 @@
         <v>439</v>
       </c>
     </row>
-    <row r="231" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="231" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B231" t="s">
         <v>435</v>
       </c>
@@ -12103,7 +12104,7 @@
         <v>439</v>
       </c>
     </row>
-    <row r="232" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="232" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B232" t="s">
         <v>441</v>
       </c>
@@ -12144,7 +12145,7 @@
         <v>444</v>
       </c>
     </row>
-    <row r="233" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="233" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B233" t="s">
         <v>441</v>
       </c>
@@ -12185,7 +12186,7 @@
         <v>444</v>
       </c>
     </row>
-    <row r="234" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="234" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B234" t="s">
         <v>441</v>
       </c>
@@ -12226,7 +12227,7 @@
         <v>444</v>
       </c>
     </row>
-    <row r="235" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="235" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B235" t="s">
         <v>441</v>
       </c>
@@ -12267,7 +12268,7 @@
         <v>444</v>
       </c>
     </row>
-    <row r="236" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="236" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B236" t="s">
         <v>441</v>
       </c>
@@ -12308,7 +12309,7 @@
         <v>452</v>
       </c>
     </row>
-    <row r="237" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="237" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B237" t="s">
         <v>441</v>
       </c>
@@ -12349,7 +12350,7 @@
         <v>452</v>
       </c>
     </row>
-    <row r="238" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="238" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B238" t="s">
         <v>441</v>
       </c>
@@ -12390,7 +12391,7 @@
         <v>452</v>
       </c>
     </row>
-    <row r="239" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="239" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B239" t="s">
         <v>441</v>
       </c>
@@ -12431,7 +12432,7 @@
         <v>452</v>
       </c>
     </row>
-    <row r="240" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="240" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B240" t="s">
         <v>400</v>
       </c>
@@ -12472,7 +12473,7 @@
         <v>458</v>
       </c>
     </row>
-    <row r="241" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="241" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B241" t="s">
         <v>400</v>
       </c>
@@ -12513,7 +12514,7 @@
         <v>458</v>
       </c>
     </row>
-    <row r="242" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="242" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B242" t="s">
         <v>400</v>
       </c>
@@ -12554,7 +12555,7 @@
         <v>463</v>
       </c>
     </row>
-    <row r="243" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="243" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B243" t="s">
         <v>400</v>
       </c>
@@ -12595,7 +12596,7 @@
         <v>463</v>
       </c>
     </row>
-    <row r="244" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="244" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B244" t="s">
         <v>400</v>
       </c>
@@ -12636,7 +12637,7 @@
         <v>463</v>
       </c>
     </row>
-    <row r="245" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="245" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B245" t="s">
         <v>400</v>
       </c>
@@ -12677,7 +12678,7 @@
         <v>463</v>
       </c>
     </row>
-    <row r="246" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="246" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B246" t="s">
         <v>467</v>
       </c>
@@ -12718,7 +12719,7 @@
         <v>471</v>
       </c>
     </row>
-    <row r="247" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="247" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B247" t="s">
         <v>467</v>
       </c>
@@ -12759,7 +12760,7 @@
         <v>471</v>
       </c>
     </row>
-    <row r="248" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="248" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B248" t="s">
         <v>473</v>
       </c>
@@ -12800,7 +12801,7 @@
         <v>478</v>
       </c>
     </row>
-    <row r="249" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="249" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B249" t="s">
         <v>473</v>
       </c>
@@ -12841,7 +12842,7 @@
         <v>478</v>
       </c>
     </row>
-    <row r="250" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="250" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B250" t="s">
         <v>184</v>
       </c>
@@ -12882,7 +12883,7 @@
         <v>483</v>
       </c>
     </row>
-    <row r="251" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="251" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B251" t="s">
         <v>484</v>
       </c>
@@ -12923,7 +12924,7 @@
         <v>489</v>
       </c>
     </row>
-    <row r="252" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="252" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B252" t="s">
         <v>484</v>
       </c>
@@ -12964,7 +12965,7 @@
         <v>489</v>
       </c>
     </row>
-    <row r="253" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="253" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B253" t="s">
         <v>473</v>
       </c>
@@ -13005,7 +13006,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="254" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="254" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B254" t="s">
         <v>473</v>
       </c>
@@ -13046,7 +13047,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="255" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="255" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B255" t="s">
         <v>495</v>
       </c>
@@ -13087,7 +13088,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="256" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="256" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B256" t="s">
         <v>196</v>
       </c>
@@ -13128,7 +13129,7 @@
         <v>504</v>
       </c>
     </row>
-    <row r="257" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="257" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B257" t="s">
         <v>226</v>
       </c>
@@ -13169,7 +13170,7 @@
         <v>508</v>
       </c>
     </row>
-    <row r="258" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="258" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B258" t="s">
         <v>226</v>
       </c>
@@ -13210,7 +13211,7 @@
         <v>508</v>
       </c>
     </row>
-    <row r="259" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="259" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B259" t="s">
         <v>510</v>
       </c>
@@ -13251,7 +13252,7 @@
         <v>514</v>
       </c>
     </row>
-    <row r="260" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="260" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B260" t="s">
         <v>515</v>
       </c>
@@ -13292,7 +13293,7 @@
         <v>519</v>
       </c>
     </row>
-    <row r="261" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="261" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B261" t="s">
         <v>520</v>
       </c>
@@ -13333,7 +13334,7 @@
         <v>525</v>
       </c>
     </row>
-    <row r="262" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="262" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B262" t="s">
         <v>345</v>
       </c>
@@ -13374,7 +13375,7 @@
         <v>528</v>
       </c>
     </row>
-    <row r="263" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="263" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B263" t="s">
         <v>345</v>
       </c>
@@ -13415,7 +13416,7 @@
         <v>528</v>
       </c>
     </row>
-    <row r="264" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="264" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B264" t="s">
         <v>345</v>
       </c>
@@ -13456,7 +13457,7 @@
         <v>528</v>
       </c>
     </row>
-    <row r="265" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="265" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B265" t="s">
         <v>345</v>
       </c>
@@ -13497,7 +13498,7 @@
         <v>528</v>
       </c>
     </row>
-    <row r="266" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="266" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B266" t="s">
         <v>520</v>
       </c>
@@ -13538,7 +13539,7 @@
         <v>534</v>
       </c>
     </row>
-    <row r="267" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="267" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B267" t="s">
         <v>520</v>
       </c>
@@ -13579,7 +13580,7 @@
         <v>534</v>
       </c>
     </row>
-    <row r="268" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="268" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B268" t="s">
         <v>520</v>
       </c>
@@ -13620,7 +13621,7 @@
         <v>534</v>
       </c>
     </row>
-    <row r="269" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="269" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B269" t="s">
         <v>106</v>
       </c>
@@ -13661,7 +13662,7 @@
         <v>539</v>
       </c>
     </row>
-    <row r="270" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="270" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B270" t="s">
         <v>106</v>
       </c>
@@ -13702,7 +13703,7 @@
         <v>539</v>
       </c>
     </row>
-    <row r="271" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="271" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B271" t="s">
         <v>106</v>
       </c>
@@ -13743,7 +13744,7 @@
         <v>539</v>
       </c>
     </row>
-    <row r="272" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="272" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B272" t="s">
         <v>106</v>
       </c>
@@ -13784,7 +13785,7 @@
         <v>539</v>
       </c>
     </row>
-    <row r="273" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="273" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B273" t="s">
         <v>69</v>
       </c>
@@ -13825,7 +13826,7 @@
         <v>545</v>
       </c>
     </row>
-    <row r="274" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="274" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B274" t="s">
         <v>546</v>
       </c>
@@ -13866,7 +13867,7 @@
         <v>550</v>
       </c>
     </row>
-    <row r="275" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="275" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B275" t="s">
         <v>546</v>
       </c>
@@ -13907,7 +13908,7 @@
         <v>550</v>
       </c>
     </row>
-    <row r="276" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="276" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B276" t="s">
         <v>546</v>
       </c>
@@ -13948,7 +13949,7 @@
         <v>550</v>
       </c>
     </row>
-    <row r="277" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="277" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B277" t="s">
         <v>520</v>
       </c>
@@ -13989,7 +13990,7 @@
         <v>556</v>
       </c>
     </row>
-    <row r="278" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="278" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B278" t="s">
         <v>441</v>
       </c>
@@ -14030,7 +14031,7 @@
         <v>560</v>
       </c>
     </row>
-    <row r="279" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="279" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B279" t="s">
         <v>441</v>
       </c>
@@ -14071,7 +14072,7 @@
         <v>560</v>
       </c>
     </row>
-    <row r="280" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="280" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B280" t="s">
         <v>441</v>
       </c>
@@ -14112,7 +14113,7 @@
         <v>560</v>
       </c>
     </row>
-    <row r="281" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="281" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B281" t="s">
         <v>515</v>
       </c>
@@ -14153,7 +14154,7 @@
         <v>565</v>
       </c>
     </row>
-    <row r="282" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="282" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B282" t="s">
         <v>515</v>
       </c>
@@ -14194,7 +14195,7 @@
         <v>565</v>
       </c>
     </row>
-    <row r="283" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="283" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B283" t="s">
         <v>515</v>
       </c>
@@ -14235,7 +14236,7 @@
         <v>565</v>
       </c>
     </row>
-    <row r="284" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="284" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B284" t="s">
         <v>515</v>
       </c>
@@ -14276,7 +14277,7 @@
         <v>565</v>
       </c>
     </row>
-    <row r="285" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="285" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B285" t="s">
         <v>515</v>
       </c>
@@ -14317,7 +14318,7 @@
         <v>565</v>
       </c>
     </row>
-    <row r="286" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="286" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B286" t="s">
         <v>520</v>
       </c>
@@ -14358,7 +14359,7 @@
         <v>573</v>
       </c>
     </row>
-    <row r="287" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="287" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B287" t="s">
         <v>574</v>
       </c>
@@ -14399,7 +14400,7 @@
         <v>578</v>
       </c>
     </row>
-    <row r="288" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="288" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B288" t="s">
         <v>579</v>
       </c>
@@ -14440,7 +14441,7 @@
         <v>583</v>
       </c>
     </row>
-    <row r="289" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="289" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B289" t="s">
         <v>579</v>
       </c>
@@ -14481,7 +14482,7 @@
         <v>583</v>
       </c>
     </row>
-    <row r="290" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="290" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B290" t="s">
         <v>585</v>
       </c>
@@ -14522,7 +14523,7 @@
         <v>589</v>
       </c>
     </row>
-    <row r="291" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="291" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B291" t="s">
         <v>590</v>
       </c>
@@ -14563,7 +14564,7 @@
         <v>594</v>
       </c>
     </row>
-    <row r="292" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="292" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B292" t="s">
         <v>400</v>
       </c>
@@ -14604,7 +14605,7 @@
         <v>597</v>
       </c>
     </row>
-    <row r="293" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="293" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B293" t="s">
         <v>400</v>
       </c>
@@ -14645,7 +14646,7 @@
         <v>597</v>
       </c>
     </row>
-    <row r="294" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="294" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B294" t="s">
         <v>585</v>
       </c>
@@ -14686,7 +14687,7 @@
         <v>601</v>
       </c>
     </row>
-    <row r="295" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="295" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B295" t="s">
         <v>585</v>
       </c>
@@ -14727,7 +14728,7 @@
         <v>601</v>
       </c>
     </row>
-    <row r="296" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="296" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B296" t="s">
         <v>366</v>
       </c>
@@ -14768,7 +14769,7 @@
         <v>605</v>
       </c>
     </row>
-    <row r="297" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="297" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B297" t="s">
         <v>579</v>
       </c>
@@ -14809,7 +14810,7 @@
         <v>609</v>
       </c>
     </row>
-    <row r="298" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="298" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B298" t="s">
         <v>590</v>
       </c>
@@ -14850,7 +14851,7 @@
         <v>612</v>
       </c>
     </row>
-    <row r="299" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="299" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B299" t="s">
         <v>590</v>
       </c>
@@ -14891,7 +14892,7 @@
         <v>612</v>
       </c>
     </row>
-    <row r="300" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="300" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B300" t="s">
         <v>495</v>
       </c>
@@ -14932,7 +14933,7 @@
         <v>616</v>
       </c>
     </row>
-    <row r="301" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="301" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B301" t="s">
         <v>467</v>
       </c>
@@ -14973,7 +14974,7 @@
         <v>620</v>
       </c>
     </row>
-    <row r="302" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="302" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B302" t="s">
         <v>473</v>
       </c>
@@ -15014,7 +15015,7 @@
         <v>623</v>
       </c>
     </row>
-    <row r="303" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="303" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B303" t="s">
         <v>473</v>
       </c>
@@ -15055,7 +15056,7 @@
         <v>623</v>
       </c>
     </row>
-    <row r="304" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="304" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B304" t="s">
         <v>473</v>
       </c>
@@ -15096,7 +15097,7 @@
         <v>623</v>
       </c>
     </row>
-    <row r="305" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="305" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B305" t="s">
         <v>473</v>
       </c>
@@ -15137,7 +15138,7 @@
         <v>623</v>
       </c>
     </row>
-    <row r="306" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="306" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B306" t="s">
         <v>226</v>
       </c>
@@ -15178,7 +15179,7 @@
         <v>630</v>
       </c>
     </row>
-    <row r="307" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="307" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B307" t="s">
         <v>226</v>
       </c>
@@ -15219,7 +15220,7 @@
         <v>630</v>
       </c>
     </row>
-    <row r="308" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="308" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B308" t="s">
         <v>366</v>
       </c>
@@ -15260,7 +15261,7 @@
         <v>634</v>
       </c>
     </row>
-    <row r="309" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="309" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B309" t="s">
         <v>366</v>
       </c>
@@ -15301,7 +15302,7 @@
         <v>634</v>
       </c>
     </row>
-    <row r="310" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="310" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B310" t="s">
         <v>366</v>
       </c>
@@ -15342,7 +15343,7 @@
         <v>634</v>
       </c>
     </row>
-    <row r="311" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="311" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B311" t="s">
         <v>637</v>
       </c>
@@ -15383,7 +15384,7 @@
         <v>641</v>
       </c>
     </row>
-    <row r="312" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="312" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B312" t="s">
         <v>637</v>
       </c>
@@ -15424,7 +15425,7 @@
         <v>641</v>
       </c>
     </row>
-    <row r="313" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="313" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B313" t="s">
         <v>643</v>
       </c>
@@ -15465,7 +15466,7 @@
         <v>647</v>
       </c>
     </row>
-    <row r="314" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="314" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B314" t="s">
         <v>643</v>
       </c>
@@ -15506,7 +15507,7 @@
         <v>647</v>
       </c>
     </row>
-    <row r="315" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="315" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B315" t="s">
         <v>574</v>
       </c>
@@ -15547,7 +15548,7 @@
         <v>651</v>
       </c>
     </row>
-    <row r="316" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="316" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B316" t="s">
         <v>574</v>
       </c>
@@ -15588,7 +15589,7 @@
         <v>651</v>
       </c>
     </row>
-    <row r="317" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="317" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B317" t="s">
         <v>637</v>
       </c>
@@ -15629,7 +15630,7 @@
         <v>655</v>
       </c>
     </row>
-    <row r="318" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="318" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B318" t="s">
         <v>106</v>
       </c>
@@ -15670,7 +15671,7 @@
         <v>659</v>
       </c>
     </row>
-    <row r="319" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="319" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B319" t="s">
         <v>106</v>
       </c>
@@ -15711,7 +15712,7 @@
         <v>659</v>
       </c>
     </row>
-    <row r="320" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="320" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B320" t="s">
         <v>106</v>
       </c>
@@ -15752,7 +15753,7 @@
         <v>659</v>
       </c>
     </row>
-    <row r="321" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="321" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B321" t="s">
         <v>257</v>
       </c>
@@ -15793,7 +15794,7 @@
         <v>664</v>
       </c>
     </row>
-    <row r="322" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="322" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B322" t="s">
         <v>395</v>
       </c>
@@ -15834,7 +15835,7 @@
         <v>667</v>
       </c>
     </row>
-    <row r="323" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="323" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B323" t="s">
         <v>395</v>
       </c>
@@ -15875,7 +15876,7 @@
         <v>667</v>
       </c>
     </row>
-    <row r="324" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="324" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B324" t="s">
         <v>395</v>
       </c>
@@ -15916,7 +15917,7 @@
         <v>667</v>
       </c>
     </row>
-    <row r="325" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="325" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B325" t="s">
         <v>395</v>
       </c>
@@ -15957,7 +15958,7 @@
         <v>667</v>
       </c>
     </row>
-    <row r="326" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="326" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B326" t="s">
         <v>395</v>
       </c>
@@ -15998,7 +15999,7 @@
         <v>667</v>
       </c>
     </row>
-    <row r="327" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="327" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B327" t="s">
         <v>395</v>
       </c>
@@ -16039,7 +16040,7 @@
         <v>667</v>
       </c>
     </row>
-    <row r="328" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="328" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B328" t="s">
         <v>395</v>
       </c>
@@ -16080,7 +16081,7 @@
         <v>667</v>
       </c>
     </row>
-    <row r="329" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="329" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B329" t="s">
         <v>579</v>
       </c>
@@ -16408,7 +16409,7 @@
         <v>679</v>
       </c>
     </row>
-    <row r="337" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="337" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B337" t="s">
         <v>435</v>
       </c>
@@ -16449,7 +16450,7 @@
         <v>689</v>
       </c>
     </row>
-    <row r="338" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="338" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B338" t="s">
         <v>435</v>
       </c>
@@ -16490,7 +16491,7 @@
         <v>689</v>
       </c>
     </row>
-    <row r="339" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="339" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B339" t="s">
         <v>585</v>
       </c>
@@ -16531,7 +16532,7 @@
         <v>694</v>
       </c>
     </row>
-    <row r="340" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="340" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B340" t="s">
         <v>695</v>
       </c>
@@ -16572,7 +16573,7 @@
         <v>700</v>
       </c>
     </row>
-    <row r="341" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="341" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B341" t="s">
         <v>701</v>
       </c>
@@ -16613,7 +16614,7 @@
         <v>706</v>
       </c>
     </row>
-    <row r="342" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="342" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B342" t="s">
         <v>93</v>
       </c>
@@ -16654,7 +16655,7 @@
         <v>709</v>
       </c>
     </row>
-    <row r="343" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="343" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B343" t="s">
         <v>710</v>
       </c>
@@ -16695,7 +16696,7 @@
         <v>714</v>
       </c>
     </row>
-    <row r="344" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="344" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B344" t="s">
         <v>643</v>
       </c>
@@ -16736,7 +16737,7 @@
         <v>717</v>
       </c>
     </row>
-    <row r="345" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="345" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B345" t="s">
         <v>643</v>
       </c>
@@ -16777,7 +16778,7 @@
         <v>721</v>
       </c>
     </row>
-    <row r="346" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="346" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B346" t="s">
         <v>643</v>
       </c>
@@ -16818,7 +16819,7 @@
         <v>721</v>
       </c>
     </row>
-    <row r="347" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="347" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B347" t="s">
         <v>643</v>
       </c>
@@ -16859,7 +16860,7 @@
         <v>721</v>
       </c>
     </row>
-    <row r="348" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="348" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B348" t="s">
         <v>643</v>
       </c>
@@ -16900,7 +16901,7 @@
         <v>721</v>
       </c>
     </row>
-    <row r="349" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="349" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B349" t="s">
         <v>643</v>
       </c>
@@ -16941,7 +16942,7 @@
         <v>721</v>
       </c>
     </row>
-    <row r="350" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="350" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B350" t="s">
         <v>93</v>
       </c>
@@ -16982,7 +16983,7 @@
         <v>729</v>
       </c>
     </row>
-    <row r="351" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="351" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B351" t="s">
         <v>93</v>
       </c>
@@ -17023,7 +17024,7 @@
         <v>729</v>
       </c>
     </row>
-    <row r="352" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="352" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B352" t="s">
         <v>366</v>
       </c>
@@ -17064,7 +17065,7 @@
         <v>733</v>
       </c>
     </row>
-    <row r="353" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="353" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B353" t="s">
         <v>366</v>
       </c>
@@ -17105,7 +17106,7 @@
         <v>733</v>
       </c>
     </row>
-    <row r="354" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="354" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B354" t="s">
         <v>366</v>
       </c>
@@ -17146,7 +17147,7 @@
         <v>733</v>
       </c>
     </row>
-    <row r="355" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="355" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B355" t="s">
         <v>484</v>
       </c>
@@ -17187,7 +17188,7 @@
         <v>738</v>
       </c>
     </row>
-    <row r="356" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="356" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B356" t="s">
         <v>484</v>
       </c>
@@ -17228,7 +17229,7 @@
         <v>738</v>
       </c>
     </row>
-    <row r="357" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="357" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B357" t="s">
         <v>484</v>
       </c>
@@ -17269,7 +17270,7 @@
         <v>738</v>
       </c>
     </row>
-    <row r="358" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="358" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B358" t="s">
         <v>741</v>
       </c>
@@ -17310,7 +17311,7 @@
         <v>745</v>
       </c>
     </row>
-    <row r="359" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="359" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B359" t="s">
         <v>741</v>
       </c>
@@ -17351,7 +17352,7 @@
         <v>745</v>
       </c>
     </row>
-    <row r="360" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="360" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B360" t="s">
         <v>360</v>
       </c>
@@ -17392,7 +17393,7 @@
         <v>750</v>
       </c>
     </row>
-    <row r="361" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="361" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B361" t="s">
         <v>701</v>
       </c>
@@ -17433,7 +17434,7 @@
         <v>753</v>
       </c>
     </row>
-    <row r="362" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="362" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B362" t="s">
         <v>710</v>
       </c>
@@ -17474,7 +17475,7 @@
         <v>756</v>
       </c>
     </row>
-    <row r="363" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="363" spans="2:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="B363" t="s">
         <v>590</v>
       </c>
@@ -17515,7 +17516,60 @@
         <v>759</v>
       </c>
     </row>
+    <row r="369" spans="9:12" x14ac:dyDescent="0.25">
+      <c r="I369" s="3">
+        <v>4407181</v>
+      </c>
+      <c r="L369" s="3">
+        <v>602393098</v>
+      </c>
+    </row>
+    <row r="370" spans="9:12" x14ac:dyDescent="0.25">
+      <c r="I370" s="3">
+        <v>4407183</v>
+      </c>
+      <c r="L370" s="3">
+        <v>602393093</v>
+      </c>
+    </row>
+    <row r="371" spans="9:12" x14ac:dyDescent="0.25">
+      <c r="I371" s="3">
+        <v>4407180</v>
+      </c>
+      <c r="L371" s="3">
+        <v>602393095</v>
+      </c>
+    </row>
+    <row r="372" spans="9:12" x14ac:dyDescent="0.25">
+      <c r="I372" s="3">
+        <v>4407179</v>
+      </c>
+      <c r="L372" s="3">
+        <v>602393092</v>
+      </c>
+    </row>
+    <row r="373" spans="9:12" x14ac:dyDescent="0.25">
+      <c r="I373" s="3">
+        <v>4407182</v>
+      </c>
+      <c r="L373" s="3">
+        <v>602393099</v>
+      </c>
+    </row>
+    <row r="374" spans="9:12" x14ac:dyDescent="0.25">
+      <c r="I374" s="3">
+        <v>4407185</v>
+      </c>
+    </row>
   </sheetData>
+  <autoFilter ref="B1:N363" xr:uid="{00000000-0001-0000-0000-000000000000}">
+    <filterColumn colId="0">
+      <filters>
+        <filter val="CIPLA"/>
+        <filter val="SUPREMEIND"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>